<commit_message>
add shunt capactors to 78L05
</commit_message>
<xml_diff>
--- a/Low noise power supply.xlsx
+++ b/Low noise power supply.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="182">
   <si>
     <t>Reference</t>
   </si>
@@ -555,6 +555,15 @@
   </si>
   <si>
     <t>nu</t>
+  </si>
+  <si>
+    <t>C40,C46,C60,C61</t>
+  </si>
+  <si>
+    <t>78L05</t>
+  </si>
+  <si>
+    <t>C60,C61 nu</t>
   </si>
 </sst>
 </file>
@@ -1129,6 +1138,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="8"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="8" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="10" xfId="10" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1140,10 +1153,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="5" xfId="10" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="8"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="8" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1526,7 +1535,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="14.4" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="8" t="s">
         <v>134</v>
       </c>
       <c r="B2" t="s">
@@ -1546,7 +1555,7 @@
       </c>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="7"/>
+      <c r="A3" s="9"/>
       <c r="B3" t="s">
         <v>7</v>
       </c>
@@ -1564,7 +1573,7 @@
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="7"/>
+      <c r="A4" s="9"/>
       <c r="B4" t="s">
         <v>129</v>
       </c>
@@ -1582,7 +1591,7 @@
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="7"/>
+      <c r="A5" s="9"/>
       <c r="B5" t="s">
         <v>130</v>
       </c>
@@ -1600,7 +1609,7 @@
       </c>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="7"/>
+      <c r="A6" s="9"/>
       <c r="B6" t="s">
         <v>34</v>
       </c>
@@ -1618,7 +1627,7 @@
       </c>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="7"/>
+      <c r="A7" s="9"/>
       <c r="B7" t="s">
         <v>44</v>
       </c>
@@ -1636,7 +1645,7 @@
       </c>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="7"/>
+      <c r="A8" s="9"/>
       <c r="B8" t="s">
         <v>48</v>
       </c>
@@ -1654,7 +1663,7 @@
       </c>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="7"/>
+      <c r="A9" s="9"/>
       <c r="B9" t="s">
         <v>52</v>
       </c>
@@ -1669,7 +1678,7 @@
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="7"/>
+      <c r="A10" s="9"/>
       <c r="B10" t="s">
         <v>59</v>
       </c>
@@ -1687,7 +1696,7 @@
       </c>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="7"/>
+      <c r="A11" s="9"/>
       <c r="B11" t="s">
         <v>62</v>
       </c>
@@ -1705,7 +1714,7 @@
       </c>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="7"/>
+      <c r="A12" s="9"/>
       <c r="B12" t="s">
         <v>66</v>
       </c>
@@ -1723,7 +1732,7 @@
       </c>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="7"/>
+      <c r="A13" s="9"/>
       <c r="B13" t="s">
         <v>70</v>
       </c>
@@ -1741,7 +1750,7 @@
       </c>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="7"/>
+      <c r="A14" s="9"/>
       <c r="B14" t="s">
         <v>74</v>
       </c>
@@ -1759,7 +1768,7 @@
       </c>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="7"/>
+      <c r="A15" s="9"/>
       <c r="B15" t="s">
         <v>77</v>
       </c>
@@ -1777,7 +1786,7 @@
       </c>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="7"/>
+      <c r="A16" s="9"/>
       <c r="B16" t="s">
         <v>80</v>
       </c>
@@ -1795,7 +1804,7 @@
       </c>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="7"/>
+      <c r="A17" s="9"/>
       <c r="B17" t="s">
         <v>132</v>
       </c>
@@ -1813,7 +1822,7 @@
       </c>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="8"/>
+      <c r="A18" s="10"/>
       <c r="B18" t="s">
         <v>113</v>
       </c>
@@ -1831,7 +1840,7 @@
       </c>
     </row>
     <row r="19" spans="1:10" ht="14.4" customHeight="1">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="11" t="s">
         <v>149</v>
       </c>
       <c r="B19" s="3" t="s">
@@ -1855,7 +1864,7 @@
       </c>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="9"/>
+      <c r="A20" s="11"/>
       <c r="B20" t="s">
         <v>136</v>
       </c>
@@ -1873,7 +1882,7 @@
       </c>
     </row>
     <row r="21" spans="1:10">
-      <c r="A21" s="9"/>
+      <c r="A21" s="11"/>
       <c r="B21" t="s">
         <v>137</v>
       </c>
@@ -1891,7 +1900,7 @@
       </c>
     </row>
     <row r="22" spans="1:10">
-      <c r="A22" s="9"/>
+      <c r="A22" s="11"/>
       <c r="B22" t="s">
         <v>18</v>
       </c>
@@ -1909,7 +1918,7 @@
       </c>
     </row>
     <row r="23" spans="1:10">
-      <c r="A23" s="9"/>
+      <c r="A23" s="11"/>
       <c r="B23" t="s">
         <v>21</v>
       </c>
@@ -1927,7 +1936,7 @@
       </c>
     </row>
     <row r="24" spans="1:10">
-      <c r="A24" s="9"/>
+      <c r="A24" s="11"/>
       <c r="B24" t="s">
         <v>146</v>
       </c>
@@ -1945,7 +1954,7 @@
       </c>
     </row>
     <row r="25" spans="1:10">
-      <c r="A25" s="9"/>
+      <c r="A25" s="11"/>
       <c r="B25" t="s">
         <v>131</v>
       </c>
@@ -1963,7 +1972,7 @@
       </c>
     </row>
     <row r="26" spans="1:10">
-      <c r="A26" s="9"/>
+      <c r="A26" s="11"/>
       <c r="B26" t="s">
         <v>138</v>
       </c>
@@ -1981,7 +1990,7 @@
       </c>
     </row>
     <row r="27" spans="1:10">
-      <c r="A27" s="9"/>
+      <c r="A27" s="11"/>
       <c r="B27" t="s">
         <v>84</v>
       </c>
@@ -1999,7 +2008,7 @@
       </c>
     </row>
     <row r="28" spans="1:10">
-      <c r="A28" s="9"/>
+      <c r="A28" s="11"/>
       <c r="B28" t="s">
         <v>139</v>
       </c>
@@ -2017,37 +2026,37 @@
       </c>
     </row>
     <row r="29" spans="1:10">
-      <c r="A29" s="9"/>
-      <c r="B29" s="10" t="s">
+      <c r="A29" s="11"/>
+      <c r="B29" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D29" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="E29" s="10" t="s">
+      <c r="E29" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="F29" s="10" t="s">
+      <c r="F29" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="G29" s="10" t="s">
+      <c r="G29" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="H29" s="10" t="s">
+      <c r="H29" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="I29" s="10">
-        <v>1</v>
-      </c>
-      <c r="J29" s="10" t="s">
+      <c r="I29" s="6">
+        <v>1</v>
+      </c>
+      <c r="J29" s="6" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:10">
-      <c r="A30" s="9"/>
+      <c r="A30" s="11"/>
       <c r="B30" t="s">
         <v>141</v>
       </c>
@@ -2065,37 +2074,37 @@
       </c>
     </row>
     <row r="31" spans="1:10">
-      <c r="A31" s="9"/>
-      <c r="B31" s="10" t="s">
+      <c r="A31" s="11"/>
+      <c r="B31" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="D31" s="10" t="s">
+      <c r="D31" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E31" s="10" t="s">
+      <c r="E31" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="F31" s="10" t="s">
+      <c r="F31" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="G31" s="11">
+      <c r="G31" s="7">
         <v>100</v>
       </c>
-      <c r="H31" s="10" t="s">
+      <c r="H31" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="I31" s="10">
-        <v>1</v>
-      </c>
-      <c r="J31" s="10" t="s">
+      <c r="I31" s="6">
+        <v>1</v>
+      </c>
+      <c r="J31" s="6" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="32" spans="1:10">
-      <c r="A32" s="9"/>
+      <c r="A32" s="11"/>
       <c r="B32" t="s">
         <v>133</v>
       </c>
@@ -2113,37 +2122,37 @@
       </c>
     </row>
     <row r="33" spans="1:10">
-      <c r="A33" s="9"/>
-      <c r="B33" s="10" t="s">
+      <c r="A33" s="11"/>
+      <c r="B33" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="D33" s="10" t="s">
+      <c r="D33" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E33" s="11">
+      <c r="E33" s="7">
         <v>909</v>
       </c>
-      <c r="F33" s="11" t="s">
+      <c r="F33" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="G33" s="11">
+      <c r="G33" s="7">
         <v>576</v>
       </c>
-      <c r="H33" s="10" t="s">
+      <c r="H33" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="I33" s="10">
-        <v>1</v>
-      </c>
-      <c r="J33" s="10" t="s">
+      <c r="I33" s="6">
+        <v>1</v>
+      </c>
+      <c r="J33" s="6" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:10">
-      <c r="A34" s="9"/>
+      <c r="A34" s="11"/>
       <c r="B34" t="s">
         <v>117</v>
       </c>
@@ -2161,7 +2170,7 @@
       </c>
     </row>
     <row r="35" spans="1:10">
-      <c r="A35" s="9"/>
+      <c r="A35" s="11"/>
       <c r="B35" t="s">
         <v>120</v>
       </c>
@@ -2179,7 +2188,7 @@
       </c>
     </row>
     <row r="36" spans="1:10">
-      <c r="A36" s="6" t="s">
+      <c r="A36" s="8" t="s">
         <v>150</v>
       </c>
       <c r="B36" s="4" t="s">
@@ -2203,7 +2212,7 @@
       </c>
     </row>
     <row r="37" spans="1:10">
-      <c r="A37" s="7"/>
+      <c r="A37" s="9"/>
       <c r="B37" t="s">
         <v>144</v>
       </c>
@@ -2221,7 +2230,7 @@
       </c>
     </row>
     <row r="38" spans="1:10">
-      <c r="A38" s="7"/>
+      <c r="A38" s="9"/>
       <c r="B38" t="s">
         <v>145</v>
       </c>
@@ -2239,7 +2248,7 @@
       </c>
     </row>
     <row r="39" spans="1:10">
-      <c r="A39" s="7"/>
+      <c r="A39" s="9"/>
       <c r="B39" t="s">
         <v>18</v>
       </c>
@@ -2257,25 +2266,33 @@
       </c>
     </row>
     <row r="40" spans="1:10">
-      <c r="A40" s="7"/>
-      <c r="B40" t="s">
-        <v>21</v>
-      </c>
-      <c r="C40" t="s">
+      <c r="A40" s="9"/>
+      <c r="B40" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C40" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="I40">
-        <v>2</v>
-      </c>
-      <c r="J40" t="s">
+      <c r="E40" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="F40" s="6"/>
+      <c r="G40" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="H40" s="6"/>
+      <c r="I40" s="6">
+        <v>4</v>
+      </c>
+      <c r="J40" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="41" spans="1:10">
-      <c r="A41" s="7"/>
+      <c r="A41" s="9"/>
       <c r="B41" t="s">
         <v>24</v>
       </c>
@@ -2293,7 +2310,7 @@
       </c>
     </row>
     <row r="42" spans="1:10">
-      <c r="A42" s="7"/>
+      <c r="A42" s="9"/>
       <c r="B42" t="s">
         <v>26</v>
       </c>
@@ -2311,7 +2328,7 @@
       </c>
     </row>
     <row r="43" spans="1:10">
-      <c r="A43" s="7"/>
+      <c r="A43" s="9"/>
       <c r="B43" t="s">
         <v>147</v>
       </c>
@@ -2329,24 +2346,24 @@
       </c>
     </row>
     <row r="44" spans="1:10">
-      <c r="A44" s="7"/>
-      <c r="B44" s="10" t="s">
+      <c r="A44" s="9"/>
+      <c r="B44" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C44" s="10" t="s">
+      <c r="C44" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D44" s="10" t="s">
+      <c r="D44" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="E44" s="10" t="s">
+      <c r="E44" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="F44" s="10"/>
-      <c r="G44" s="10" t="s">
+      <c r="F44" s="6"/>
+      <c r="G44" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="H44" s="10"/>
+      <c r="H44" s="6"/>
       <c r="I44">
         <v>1</v>
       </c>
@@ -2355,7 +2372,7 @@
       </c>
     </row>
     <row r="45" spans="1:10">
-      <c r="A45" s="7"/>
+      <c r="A45" s="9"/>
       <c r="B45" t="s">
         <v>40</v>
       </c>
@@ -2373,7 +2390,7 @@
       </c>
     </row>
     <row r="46" spans="1:10">
-      <c r="A46" s="7"/>
+      <c r="A46" s="9"/>
       <c r="B46" t="s">
         <v>148</v>
       </c>
@@ -2391,7 +2408,7 @@
       </c>
     </row>
     <row r="47" spans="1:10">
-      <c r="A47" s="7"/>
+      <c r="A47" s="9"/>
       <c r="B47" t="s">
         <v>56</v>
       </c>
@@ -2409,7 +2426,7 @@
       </c>
     </row>
     <row r="48" spans="1:10">
-      <c r="A48" s="7"/>
+      <c r="A48" s="9"/>
       <c r="B48" t="s">
         <v>84</v>
       </c>
@@ -2427,7 +2444,7 @@
       </c>
     </row>
     <row r="49" spans="1:10">
-      <c r="A49" s="7"/>
+      <c r="A49" s="9"/>
       <c r="B49" t="s">
         <v>139</v>
       </c>
@@ -2445,37 +2462,37 @@
       </c>
     </row>
     <row r="50" spans="1:10">
-      <c r="A50" s="7"/>
-      <c r="B50" s="10" t="s">
+      <c r="A50" s="9"/>
+      <c r="B50" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="C50" s="10" t="s">
+      <c r="C50" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="D50" s="10" t="s">
+      <c r="D50" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="E50" s="10" t="s">
+      <c r="E50" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="F50" s="10" t="s">
+      <c r="F50" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="G50" s="10" t="s">
+      <c r="G50" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="H50" s="10" t="s">
+      <c r="H50" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="I50" s="10">
-        <v>1</v>
-      </c>
-      <c r="J50" s="10" t="s">
+      <c r="I50" s="6">
+        <v>1</v>
+      </c>
+      <c r="J50" s="6" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="51" spans="1:10">
-      <c r="A51" s="7"/>
+      <c r="A51" s="9"/>
       <c r="B51" t="s">
         <v>141</v>
       </c>
@@ -2493,37 +2510,37 @@
       </c>
     </row>
     <row r="52" spans="1:10">
-      <c r="A52" s="7"/>
-      <c r="B52" s="10" t="s">
+      <c r="A52" s="9"/>
+      <c r="B52" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="C52" s="10" t="s">
+      <c r="C52" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="D52" s="10" t="s">
+      <c r="D52" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E52" s="10" t="s">
+      <c r="E52" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="F52" s="10" t="s">
+      <c r="F52" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="G52" s="11">
+      <c r="G52" s="7">
         <v>100</v>
       </c>
-      <c r="H52" s="10" t="s">
+      <c r="H52" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="I52" s="10">
-        <v>1</v>
-      </c>
-      <c r="J52" s="10" t="s">
+      <c r="I52" s="6">
+        <v>1</v>
+      </c>
+      <c r="J52" s="6" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="53" spans="1:10">
-      <c r="A53" s="7"/>
+      <c r="A53" s="9"/>
       <c r="B53" t="s">
         <v>140</v>
       </c>
@@ -2541,7 +2558,7 @@
       </c>
     </row>
     <row r="54" spans="1:10">
-      <c r="A54" s="7"/>
+      <c r="A54" s="9"/>
       <c r="B54" t="s">
         <v>142</v>
       </c>
@@ -2559,7 +2576,7 @@
       </c>
     </row>
     <row r="55" spans="1:10">
-      <c r="A55" s="7"/>
+      <c r="A55" s="9"/>
       <c r="B55" t="s">
         <v>101</v>
       </c>
@@ -2577,97 +2594,97 @@
       </c>
     </row>
     <row r="56" spans="1:10">
-      <c r="A56" s="7"/>
-      <c r="B56" s="10" t="s">
+      <c r="A56" s="9"/>
+      <c r="B56" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="C56" s="10" t="s">
+      <c r="C56" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="D56" s="10" t="s">
+      <c r="D56" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="E56" s="10" t="s">
+      <c r="E56" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="F56" s="10" t="s">
+      <c r="F56" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="G56" s="10" t="s">
+      <c r="G56" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="H56" s="10" t="s">
+      <c r="H56" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="I56" s="10">
-        <v>1</v>
-      </c>
-      <c r="J56" s="10" t="s">
+      <c r="I56" s="6">
+        <v>1</v>
+      </c>
+      <c r="J56" s="6" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="57" spans="1:10">
-      <c r="A57" s="7"/>
-      <c r="B57" s="10" t="s">
+      <c r="A57" s="9"/>
+      <c r="B57" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="C57" s="10" t="s">
+      <c r="C57" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="D57" s="10" t="s">
+      <c r="D57" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="E57" s="10" t="s">
+      <c r="E57" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="F57" s="10" t="s">
+      <c r="F57" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="G57" s="10" t="s">
+      <c r="G57" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="H57" s="10" t="s">
+      <c r="H57" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="I57" s="10">
-        <v>1</v>
-      </c>
-      <c r="J57" s="10" t="s">
+      <c r="I57" s="6">
+        <v>1</v>
+      </c>
+      <c r="J57" s="6" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="58" spans="1:10">
-      <c r="A58" s="7"/>
-      <c r="B58" s="10" t="s">
+      <c r="A58" s="9"/>
+      <c r="B58" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="C58" s="10" t="s">
+      <c r="C58" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="D58" s="10" t="s">
+      <c r="D58" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="E58" s="10" t="s">
+      <c r="E58" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="F58" s="10" t="s">
+      <c r="F58" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="G58" s="10" t="s">
+      <c r="G58" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="H58" s="10" t="s">
+      <c r="H58" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="I58" s="10">
-        <v>1</v>
-      </c>
-      <c r="J58" s="10" t="s">
+      <c r="I58" s="6">
+        <v>1</v>
+      </c>
+      <c r="J58" s="6" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="59" spans="1:10">
-      <c r="A59" s="7"/>
+      <c r="A59" s="9"/>
       <c r="B59" t="s">
         <v>117</v>
       </c>
@@ -2685,24 +2702,24 @@
       </c>
     </row>
     <row r="60" spans="1:10">
-      <c r="A60" s="7"/>
-      <c r="B60" s="10" t="s">
+      <c r="A60" s="9"/>
+      <c r="B60" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C60" s="10" t="s">
-        <v>124</v>
-      </c>
-      <c r="D60" s="10" t="s">
-        <v>124</v>
-      </c>
-      <c r="E60" s="10" t="s">
+      <c r="C60" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="E60" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="F60" s="10"/>
-      <c r="G60" s="10" t="s">
+      <c r="F60" s="6"/>
+      <c r="G60" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="H60" s="10"/>
+      <c r="H60" s="6"/>
       <c r="I60">
         <v>1</v>
       </c>
@@ -2711,7 +2728,7 @@
       </c>
     </row>
     <row r="61" spans="1:10">
-      <c r="A61" s="8"/>
+      <c r="A61" s="10"/>
       <c r="B61" t="s">
         <v>126</v>
       </c>

</xml_diff>

<commit_message>
new power stage output 3V3 2A
</commit_message>
<xml_diff>
--- a/Low noise power supply.xlsx
+++ b/Low noise power supply.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="188">
   <si>
     <t>Reference</t>
   </si>
@@ -564,6 +564,24 @@
   </si>
   <si>
     <t>C60,C61 nu</t>
+  </si>
+  <si>
+    <t>R22,R23</t>
+  </si>
+  <si>
+    <t>470k</t>
+  </si>
+  <si>
+    <t>RC1206FR-07470KL</t>
+  </si>
+  <si>
+    <t>C62</t>
+  </si>
+  <si>
+    <t>2n2</t>
+  </si>
+  <si>
+    <t>CC1206KKX7RZBB222</t>
   </si>
 </sst>
 </file>
@@ -1489,7 +1507,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J63"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="22.21875" customWidth="1"/>
@@ -1593,193 +1611,193 @@
     <row r="5" spans="1:10">
       <c r="A5" s="9"/>
       <c r="B5" t="s">
-        <v>130</v>
+        <v>185</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>186</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>187</v>
       </c>
       <c r="I5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="9"/>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>130</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="9"/>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="I7">
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="9"/>
       <c r="B8" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I8">
         <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="9"/>
       <c r="B9" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D9" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="I9">
         <v>1</v>
+      </c>
+      <c r="J9" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="9"/>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C10" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="D10" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="I10">
         <v>1</v>
-      </c>
-      <c r="J10" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="9"/>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D11" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="9"/>
       <c r="B12" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D12" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="I12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J12" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="9"/>
       <c r="B13" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C13" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D13" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="I13">
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="9"/>
       <c r="B14" t="s">
-        <v>74</v>
-      </c>
-      <c r="C14" s="2">
-        <v>750</v>
+        <v>70</v>
+      </c>
+      <c r="C14" t="s">
+        <v>71</v>
       </c>
       <c r="D14" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I14">
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="9"/>
       <c r="B15" t="s">
-        <v>77</v>
-      </c>
-      <c r="C15" t="s">
-        <v>78</v>
+        <v>74</v>
+      </c>
+      <c r="C15" s="2">
+        <v>750</v>
       </c>
       <c r="D15" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="I15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J15" t="s">
         <v>76</v>
@@ -1788,16 +1806,16 @@
     <row r="16" spans="1:10">
       <c r="A16" s="9"/>
       <c r="B16" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C16" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D16" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J16" t="s">
         <v>76</v>
@@ -1806,112 +1824,112 @@
     <row r="17" spans="1:10">
       <c r="A17" s="9"/>
       <c r="B17" t="s">
-        <v>132</v>
-      </c>
-      <c r="C17" s="2">
-        <v>240</v>
+        <v>80</v>
+      </c>
+      <c r="C17" t="s">
+        <v>81</v>
       </c>
       <c r="D17" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J17" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="10"/>
+      <c r="A18" s="9"/>
       <c r="B18" t="s">
+        <v>132</v>
+      </c>
+      <c r="C18" s="2">
+        <v>240</v>
+      </c>
+      <c r="D18" t="s">
+        <v>83</v>
+      </c>
+      <c r="I18">
+        <v>2</v>
+      </c>
+      <c r="J18" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10">
+      <c r="A19" s="9"/>
+      <c r="B19" t="s">
+        <v>182</v>
+      </c>
+      <c r="C19" t="s">
+        <v>183</v>
+      </c>
+      <c r="D19" t="s">
+        <v>184</v>
+      </c>
+      <c r="I19">
+        <v>2</v>
+      </c>
+      <c r="J19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10">
+      <c r="A20" s="10"/>
+      <c r="B20" t="s">
         <v>113</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C20" t="s">
         <v>114</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D20" t="s">
         <v>115</v>
       </c>
-      <c r="I18">
-        <v>1</v>
-      </c>
-      <c r="J18" t="s">
+      <c r="I20">
+        <v>1</v>
+      </c>
+      <c r="J20" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="14.4" customHeight="1">
-      <c r="A19" s="11" t="s">
+    <row r="21" spans="1:10" ht="14.4" customHeight="1">
+      <c r="A21" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B21" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C21" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D21" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4">
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4">
         <v>4</v>
       </c>
-      <c r="J19" s="4" t="s">
+      <c r="J21" s="4" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10">
-      <c r="A20" s="11"/>
-      <c r="B20" t="s">
-        <v>136</v>
-      </c>
-      <c r="C20" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" t="s">
-        <v>11</v>
-      </c>
-      <c r="I20">
-        <v>2</v>
-      </c>
-      <c r="J20" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10">
-      <c r="A21" s="11"/>
-      <c r="B21" t="s">
-        <v>137</v>
-      </c>
-      <c r="C21" t="s">
-        <v>15</v>
-      </c>
-      <c r="D21" t="s">
-        <v>16</v>
-      </c>
-      <c r="I21">
-        <v>5</v>
-      </c>
-      <c r="J21" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="11"/>
       <c r="B22" t="s">
-        <v>18</v>
+        <v>136</v>
       </c>
       <c r="C22" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="D22" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="I22">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J22" t="s">
         <v>12</v>
@@ -1920,16 +1938,16 @@
     <row r="23" spans="1:10">
       <c r="A23" s="11"/>
       <c r="B23" t="s">
-        <v>21</v>
+        <v>137</v>
       </c>
       <c r="C23" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D23" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="I23">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J23" t="s">
         <v>17</v>
@@ -1938,133 +1956,121 @@
     <row r="24" spans="1:10">
       <c r="A24" s="11"/>
       <c r="B24" t="s">
-        <v>146</v>
+        <v>18</v>
       </c>
       <c r="C24" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="D24" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="I24">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J24" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="11"/>
       <c r="B25" t="s">
-        <v>131</v>
+        <v>21</v>
       </c>
       <c r="C25" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D25" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J25" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="11"/>
       <c r="B26" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="C26" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="D26" t="s">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J26" t="s">
-        <v>55</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="11"/>
       <c r="B27" t="s">
-        <v>84</v>
+        <v>131</v>
       </c>
       <c r="C27" t="s">
-        <v>85</v>
+        <v>32</v>
       </c>
       <c r="D27" t="s">
-        <v>86</v>
+        <v>32</v>
       </c>
       <c r="I27">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J27" t="s">
-        <v>87</v>
+        <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="11"/>
       <c r="B28" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C28" t="s">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="D28" t="s">
-        <v>89</v>
+        <v>54</v>
       </c>
       <c r="I28">
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="11"/>
-      <c r="B29" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G29" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="H29" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="I29" s="6">
-        <v>1</v>
-      </c>
-      <c r="J29" s="6" t="s">
-        <v>76</v>
+      <c r="B29" t="s">
+        <v>84</v>
+      </c>
+      <c r="C29" t="s">
+        <v>85</v>
+      </c>
+      <c r="D29" t="s">
+        <v>86</v>
+      </c>
+      <c r="I29">
+        <v>2</v>
+      </c>
+      <c r="J29" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="11"/>
       <c r="B30" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C30" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D30" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="I30">
         <v>1</v>
@@ -2076,25 +2082,25 @@
     <row r="31" spans="1:10">
       <c r="A31" s="11"/>
       <c r="B31" s="6" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>155</v>
+        <v>88</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="G31" s="7">
-        <v>100</v>
+        <v>89</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>154</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="I31" s="6">
         <v>1</v>
@@ -2106,13 +2112,13 @@
     <row r="32" spans="1:10">
       <c r="A32" s="11"/>
       <c r="B32" t="s">
-        <v>133</v>
-      </c>
-      <c r="C32" s="2">
-        <v>240</v>
+        <v>141</v>
+      </c>
+      <c r="C32" t="s">
+        <v>93</v>
       </c>
       <c r="D32" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="I32">
         <v>1</v>
@@ -2124,25 +2130,25 @@
     <row r="33" spans="1:10">
       <c r="A33" s="11"/>
       <c r="B33" s="6" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D33" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="G33" s="7">
         <v>100</v>
       </c>
-      <c r="E33" s="7">
-        <v>909</v>
-      </c>
-      <c r="F33" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="G33" s="7">
-        <v>576</v>
-      </c>
       <c r="H33" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="I33" s="6">
         <v>1</v>
@@ -2154,112 +2160,124 @@
     <row r="34" spans="1:10">
       <c r="A34" s="11"/>
       <c r="B34" t="s">
-        <v>117</v>
-      </c>
-      <c r="C34" t="s">
-        <v>118</v>
+        <v>133</v>
+      </c>
+      <c r="C34" s="2">
+        <v>240</v>
       </c>
       <c r="D34" t="s">
-        <v>118</v>
+        <v>83</v>
       </c>
       <c r="I34">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>119</v>
+        <v>76</v>
       </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="11"/>
-      <c r="B35" t="s">
+      <c r="B35" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E35" s="7">
+        <v>909</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="G35" s="7">
+        <v>576</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="I35" s="6">
+        <v>1</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10">
+      <c r="A36" s="11"/>
+      <c r="B36" t="s">
+        <v>117</v>
+      </c>
+      <c r="C36" t="s">
+        <v>118</v>
+      </c>
+      <c r="D36" t="s">
+        <v>118</v>
+      </c>
+      <c r="I36">
+        <v>2</v>
+      </c>
+      <c r="J36" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10">
+      <c r="A37" s="11"/>
+      <c r="B37" t="s">
         <v>120</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C37" t="s">
         <v>121</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D37" t="s">
         <v>121</v>
       </c>
-      <c r="I35">
-        <v>1</v>
-      </c>
-      <c r="J35" t="s">
+      <c r="I37">
+        <v>1</v>
+      </c>
+      <c r="J37" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="36" spans="1:10">
-      <c r="A36" s="8" t="s">
+    <row r="38" spans="1:10">
+      <c r="A38" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B38" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="C38" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D36" s="4" t="s">
+      <c r="D38" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
-      <c r="I36" s="4">
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="4"/>
+      <c r="I38" s="4">
         <v>4</v>
       </c>
-      <c r="J36" s="4" t="s">
+      <c r="J38" s="4" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10">
-      <c r="A37" s="9"/>
-      <c r="B37" t="s">
-        <v>144</v>
-      </c>
-      <c r="C37" t="s">
-        <v>10</v>
-      </c>
-      <c r="D37" t="s">
-        <v>11</v>
-      </c>
-      <c r="I37">
-        <v>2</v>
-      </c>
-      <c r="J37" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10">
-      <c r="A38" s="9"/>
-      <c r="B38" t="s">
-        <v>145</v>
-      </c>
-      <c r="C38" t="s">
-        <v>15</v>
-      </c>
-      <c r="D38" t="s">
-        <v>16</v>
-      </c>
-      <c r="I38">
-        <v>6</v>
-      </c>
-      <c r="J38" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="9"/>
       <c r="B39" t="s">
-        <v>18</v>
+        <v>144</v>
       </c>
       <c r="C39" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="D39" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="I39">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J39" t="s">
         <v>12</v>
@@ -2267,240 +2285,228 @@
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="9"/>
-      <c r="B40" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D40" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="F40" s="6"/>
-      <c r="G40" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="H40" s="6"/>
-      <c r="I40" s="6">
-        <v>4</v>
-      </c>
-      <c r="J40" s="6" t="s">
+      <c r="B40" t="s">
+        <v>145</v>
+      </c>
+      <c r="C40" t="s">
+        <v>15</v>
+      </c>
+      <c r="D40" t="s">
+        <v>16</v>
+      </c>
+      <c r="I40">
+        <v>6</v>
+      </c>
+      <c r="J40" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="9"/>
       <c r="B41" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C41" t="s">
+        <v>19</v>
+      </c>
+      <c r="D41" t="s">
+        <v>20</v>
+      </c>
+      <c r="I41">
         <v>4</v>
       </c>
-      <c r="D41" t="s">
-        <v>25</v>
-      </c>
-      <c r="I41">
-        <v>1</v>
-      </c>
       <c r="J41" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" s="9"/>
-      <c r="B42" t="s">
-        <v>26</v>
-      </c>
-      <c r="C42" t="s">
-        <v>27</v>
-      </c>
-      <c r="D42" t="s">
-        <v>28</v>
-      </c>
-      <c r="I42">
-        <v>1</v>
-      </c>
-      <c r="J42" t="s">
+      <c r="B42" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="F42" s="6"/>
+      <c r="G42" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="H42" s="6"/>
+      <c r="I42" s="6">
+        <v>4</v>
+      </c>
+      <c r="J42" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="9"/>
       <c r="B43" t="s">
-        <v>147</v>
+        <v>24</v>
       </c>
       <c r="C43" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D43" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="I43">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J43" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
     </row>
     <row r="44" spans="1:10">
       <c r="A44" s="9"/>
-      <c r="B44" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="F44" s="6"/>
-      <c r="G44" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="H44" s="6"/>
+      <c r="B44" t="s">
+        <v>26</v>
+      </c>
+      <c r="C44" t="s">
+        <v>27</v>
+      </c>
+      <c r="D44" t="s">
+        <v>28</v>
+      </c>
       <c r="I44">
         <v>1</v>
       </c>
       <c r="J44" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
     </row>
     <row r="45" spans="1:10">
       <c r="A45" s="9"/>
       <c r="B45" t="s">
-        <v>40</v>
+        <v>147</v>
       </c>
       <c r="C45" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="D45" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="I45">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J45" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" s="9"/>
-      <c r="B46" t="s">
-        <v>148</v>
-      </c>
-      <c r="C46" t="s">
-        <v>19</v>
-      </c>
-      <c r="D46" t="s">
-        <v>54</v>
-      </c>
+      <c r="B46" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="F46" s="6"/>
+      <c r="G46" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="H46" s="6"/>
       <c r="I46">
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" s="9"/>
       <c r="B47" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="C47" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="D47" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="I47">
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
     </row>
     <row r="48" spans="1:10">
       <c r="A48" s="9"/>
       <c r="B48" t="s">
-        <v>84</v>
+        <v>148</v>
       </c>
       <c r="C48" t="s">
-        <v>85</v>
+        <v>19</v>
       </c>
       <c r="D48" t="s">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="I48">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>87</v>
+        <v>55</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="9"/>
       <c r="B49" t="s">
-        <v>139</v>
+        <v>56</v>
       </c>
       <c r="C49" t="s">
-        <v>88</v>
+        <v>57</v>
       </c>
       <c r="D49" t="s">
-        <v>89</v>
+        <v>58</v>
       </c>
       <c r="I49">
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="9"/>
-      <c r="B50" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="F50" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G50" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="H50" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="I50" s="6">
-        <v>1</v>
-      </c>
-      <c r="J50" s="6" t="s">
-        <v>76</v>
+      <c r="B50" t="s">
+        <v>84</v>
+      </c>
+      <c r="C50" t="s">
+        <v>85</v>
+      </c>
+      <c r="D50" t="s">
+        <v>86</v>
+      </c>
+      <c r="I50">
+        <v>2</v>
+      </c>
+      <c r="J50" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="51" spans="1:10">
       <c r="A51" s="9"/>
       <c r="B51" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C51" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D51" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="I51">
         <v>1</v>
@@ -2512,25 +2518,25 @@
     <row r="52" spans="1:10">
       <c r="A52" s="9"/>
       <c r="B52" s="6" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>155</v>
+        <v>88</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="G52" s="7">
-        <v>100</v>
+        <v>89</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>154</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="I52" s="6">
         <v>1</v>
@@ -2542,13 +2548,13 @@
     <row r="53" spans="1:10">
       <c r="A53" s="9"/>
       <c r="B53" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C53" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D53" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="I53">
         <v>1</v>
@@ -2559,32 +2565,44 @@
     </row>
     <row r="54" spans="1:10">
       <c r="A54" s="9"/>
-      <c r="B54" t="s">
-        <v>142</v>
-      </c>
-      <c r="C54" t="s">
-        <v>93</v>
-      </c>
-      <c r="D54" t="s">
-        <v>94</v>
-      </c>
-      <c r="I54">
-        <v>1</v>
-      </c>
-      <c r="J54" t="s">
+      <c r="B54" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="G54" s="7">
+        <v>100</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="I54" s="6">
+        <v>1</v>
+      </c>
+      <c r="J54" s="6" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="55" spans="1:10">
       <c r="A55" s="9"/>
       <c r="B55" t="s">
-        <v>101</v>
+        <v>140</v>
       </c>
       <c r="C55" t="s">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="D55" t="s">
-        <v>103</v>
+        <v>89</v>
       </c>
       <c r="I55">
         <v>1</v>
@@ -2595,86 +2613,62 @@
     </row>
     <row r="56" spans="1:10">
       <c r="A56" s="9"/>
-      <c r="B56" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="D56" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="F56" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="G56" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="H56" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="I56" s="6">
-        <v>1</v>
-      </c>
-      <c r="J56" s="6" t="s">
+      <c r="B56" t="s">
+        <v>142</v>
+      </c>
+      <c r="C56" t="s">
+        <v>93</v>
+      </c>
+      <c r="D56" t="s">
+        <v>94</v>
+      </c>
+      <c r="I56">
+        <v>1</v>
+      </c>
+      <c r="J56" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="57" spans="1:10">
       <c r="A57" s="9"/>
-      <c r="B57" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="D57" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="E57" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="F57" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="G57" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="H57" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="I57" s="6">
-        <v>1</v>
-      </c>
-      <c r="J57" s="6" t="s">
+      <c r="B57" t="s">
+        <v>101</v>
+      </c>
+      <c r="C57" t="s">
+        <v>102</v>
+      </c>
+      <c r="D57" t="s">
+        <v>103</v>
+      </c>
+      <c r="I57">
+        <v>1</v>
+      </c>
+      <c r="J57" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="58" spans="1:10">
       <c r="A58" s="9"/>
       <c r="B58" s="6" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="I58" s="6">
         <v>1</v>
@@ -2685,71 +2679,131 @@
     </row>
     <row r="59" spans="1:10">
       <c r="A59" s="9"/>
-      <c r="B59" t="s">
-        <v>117</v>
-      </c>
-      <c r="C59" t="s">
-        <v>118</v>
-      </c>
-      <c r="D59" t="s">
-        <v>118</v>
-      </c>
-      <c r="I59">
-        <v>2</v>
-      </c>
-      <c r="J59" t="s">
-        <v>119</v>
+      <c r="B59" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="F59" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="I59" s="6">
+        <v>1</v>
+      </c>
+      <c r="J59" s="6" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="60" spans="1:10">
       <c r="A60" s="9"/>
       <c r="B60" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="G60" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="H60" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="I60" s="6">
+        <v>1</v>
+      </c>
+      <c r="J60" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10">
+      <c r="A61" s="9"/>
+      <c r="B61" t="s">
+        <v>117</v>
+      </c>
+      <c r="C61" t="s">
+        <v>118</v>
+      </c>
+      <c r="D61" t="s">
+        <v>118</v>
+      </c>
+      <c r="I61">
+        <v>2</v>
+      </c>
+      <c r="J61" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10">
+      <c r="A62" s="9"/>
+      <c r="B62" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C60" s="6" t="s">
+      <c r="C62" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D60" s="6" t="s">
+      <c r="D62" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="E60" s="6" t="s">
+      <c r="E62" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="F60" s="6"/>
-      <c r="G60" s="6" t="s">
+      <c r="F62" s="6"/>
+      <c r="G62" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="H60" s="6"/>
-      <c r="I60">
-        <v>1</v>
-      </c>
-      <c r="J60" t="s">
+      <c r="H62" s="6"/>
+      <c r="I62">
+        <v>1</v>
+      </c>
+      <c r="J62" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="61" spans="1:10">
-      <c r="A61" s="10"/>
-      <c r="B61" t="s">
+    <row r="63" spans="1:10">
+      <c r="A63" s="10"/>
+      <c r="B63" t="s">
         <v>126</v>
       </c>
-      <c r="C61" t="s">
+      <c r="C63" t="s">
         <v>127</v>
       </c>
-      <c r="D61" t="s">
+      <c r="D63" t="s">
         <v>127</v>
       </c>
-      <c r="I61">
-        <v>1</v>
-      </c>
-      <c r="J61" t="s">
+      <c r="I63">
+        <v>1</v>
+      </c>
+      <c r="J63" t="s">
         <v>128</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:A18"/>
-    <mergeCell ref="A19:A35"/>
-    <mergeCell ref="A36:A61"/>
+    <mergeCell ref="A2:A20"/>
+    <mergeCell ref="A21:A37"/>
+    <mergeCell ref="A38:A63"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1">

</xml_diff>